<commit_message>
Actualizar cache, DWLT, pronostico, historico y validacion Loreto
</commit_message>
<xml_diff>
--- a/outputs/metricas_dwlt_estaciones.xlsx
+++ b/outputs/metricas_dwlt_estaciones.xlsx
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E2" t="n">
         <v>10026</v>
@@ -582,7 +582,7 @@
         <v>10</v>
       </c>
       <c r="G2" t="n">
-        <v>10025</v>
+        <v>10026</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -599,13 +599,13 @@
         <v>36161</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M2" t="n">
         <v>1.78</v>
       </c>
       <c r="N2" t="n">
-        <v>102.6205066001663</v>
+        <v>102.610656160649</v>
       </c>
       <c r="O2" t="n">
         <v>118.97</v>
@@ -614,37 +614,37 @@
         <v>1.843123209169055</v>
       </c>
       <c r="Q2" t="n">
-        <v>102.5931657179678</v>
+        <v>102.5896691920469</v>
       </c>
       <c r="R2" t="n">
         <v>118.8919225199131</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.02734088219847836</v>
+        <v>-0.02098696860207732</v>
       </c>
       <c r="T2" t="n">
-        <v>17.91768909780116</v>
+        <v>17.9155038668804</v>
       </c>
       <c r="U2" t="n">
-        <v>36.0553248564454</v>
+        <v>36.05009345612843</v>
       </c>
       <c r="V2" t="n">
-        <v>0.1401580122222274</v>
+        <v>0.1409931890664702</v>
       </c>
       <c r="W2" t="n">
-        <v>-0.7185017679962451</v>
+        <v>-0.7159677077673274</v>
       </c>
       <c r="X2" t="n">
-        <v>0.1401576954494871</v>
+        <v>0.1409923376428469</v>
       </c>
       <c r="Y2" t="n">
-        <v>2.975828943454343</v>
+        <v>2.975681600135594</v>
       </c>
       <c r="Z2" t="n">
-        <v>80.91433054852874</v>
+        <v>95.02088030319564</v>
       </c>
       <c r="AA2" t="n">
-        <v>110.2664412526513</v>
+        <v>111.56</v>
       </c>
     </row>
     <row r="3">
@@ -662,16 +662,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E3" t="n">
+        <v>14621</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" t="n">
         <v>14620</v>
-      </c>
-      <c r="F3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G3" t="n">
-        <v>14619</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -688,13 +688,13 @@
         <v>30317</v>
       </c>
       <c r="L3" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M3" t="n">
         <v>0.01</v>
       </c>
       <c r="N3" t="n">
-        <v>4.908950954237636</v>
+        <v>4.908743604651163</v>
       </c>
       <c r="O3" t="n">
         <v>11.07</v>
@@ -703,37 +703,37 @@
         <v>0.01</v>
       </c>
       <c r="Q3" t="n">
-        <v>4.966491300692143</v>
+        <v>4.966298123086359</v>
       </c>
       <c r="R3" t="n">
         <v>11.07</v>
       </c>
       <c r="S3" t="n">
-        <v>0.05754034645450718</v>
+        <v>0.05755451843519679</v>
       </c>
       <c r="T3" t="n">
-        <v>1.344678651577674</v>
+        <v>1.344604257897916</v>
       </c>
       <c r="U3" t="n">
-        <v>1.719196561490579</v>
+        <v>1.719132378703679</v>
       </c>
       <c r="V3" t="n">
-        <v>0.7813193129006681</v>
+        <v>0.7813394727654076</v>
       </c>
       <c r="W3" t="n">
-        <v>0.5696226494754484</v>
+        <v>0.5696647336036537</v>
       </c>
       <c r="X3" t="n">
-        <v>0.7802836051556702</v>
+        <v>0.7803029433525255</v>
       </c>
       <c r="Y3" t="n">
-        <v>2.150881791483113</v>
+        <v>2.089206338985151</v>
       </c>
       <c r="Z3" t="n">
-        <v>2.225661007061721</v>
+        <v>2.207129567189043</v>
       </c>
       <c r="AA3" t="n">
-        <v>2.331233021292217</v>
+        <v>2.330687820983126</v>
       </c>
     </row>
     <row r="4">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E4" t="n">
         <v>10253</v>
@@ -792,37 +792,37 @@
         <v>0.3676769446391031</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.239112466735863</v>
+        <v>7.239024853385637</v>
       </c>
       <c r="R4" t="n">
         <v>12.72990889978977</v>
       </c>
       <c r="S4" t="n">
-        <v>0.3294513919284887</v>
+        <v>0.3293637785782629</v>
       </c>
       <c r="T4" t="n">
-        <v>1.292410023992817</v>
+        <v>1.292382973225675</v>
       </c>
       <c r="U4" t="n">
-        <v>1.682184810210951</v>
+        <v>1.682164199629526</v>
       </c>
       <c r="V4" t="n">
-        <v>0.8676885492328213</v>
+        <v>0.8676924368946518</v>
       </c>
       <c r="W4" t="n">
-        <v>0.737547182802971</v>
+        <v>0.7375536140487986</v>
       </c>
       <c r="X4" t="n">
-        <v>0.8472055693195504</v>
+        <v>0.8472296644216341</v>
       </c>
       <c r="Y4" t="n">
-        <v>3.181960352422907</v>
+        <v>3.180150403521643</v>
       </c>
       <c r="Z4" t="n">
-        <v>3.304003187825538</v>
+        <v>3.456767148899859</v>
       </c>
       <c r="AA4" t="n">
-        <v>3.496518272400334</v>
+        <v>3.968782098312546</v>
       </c>
     </row>
     <row r="5">
@@ -840,7 +840,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E5" t="n">
         <v>2710</v>
@@ -878,40 +878,40 @@
         <v>15.51</v>
       </c>
       <c r="P5" t="n">
-        <v>2.75798825256975</v>
+        <v>2.757769625825385</v>
       </c>
       <c r="Q5" t="n">
-        <v>9.302284779643362</v>
+        <v>9.30216591702032</v>
       </c>
       <c r="R5" t="n">
         <v>15.38127820602663</v>
       </c>
       <c r="S5" t="n">
-        <v>0.3609821966175324</v>
+        <v>0.3608633339944894</v>
       </c>
       <c r="T5" t="n">
-        <v>1.253989156906</v>
+        <v>1.254014140263419</v>
       </c>
       <c r="U5" t="n">
-        <v>1.750199988890713</v>
+        <v>1.750208620978122</v>
       </c>
       <c r="V5" t="n">
-        <v>0.866204813272385</v>
+        <v>0.8662064762243523</v>
       </c>
       <c r="W5" t="n">
-        <v>0.721294252761383</v>
+        <v>0.7212915035689254</v>
       </c>
       <c r="X5" t="n">
-        <v>0.8602183440303083</v>
+        <v>0.8602248242357605</v>
       </c>
       <c r="Y5" t="n">
-        <v>4.871414572875782</v>
+        <v>4.776907411505261</v>
       </c>
       <c r="Z5" t="n">
-        <v>5.19583926257148</v>
+        <v>5.194475984089943</v>
       </c>
       <c r="AA5" t="n">
-        <v>5.726413692731685</v>
+        <v>5.807229304175822</v>
       </c>
     </row>
     <row r="6">
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E6" t="n">
         <v>8866</v>
@@ -970,37 +970,37 @@
         <v>1.616683937823834</v>
       </c>
       <c r="Q6" t="n">
-        <v>7.022006934507797</v>
+        <v>7.021977346764491</v>
       </c>
       <c r="R6" t="n">
         <v>10.19050035038543</v>
       </c>
       <c r="S6" t="n">
-        <v>0.2883830906097593</v>
+        <v>0.2883535028664529</v>
       </c>
       <c r="T6" t="n">
-        <v>1.479832553395997</v>
+        <v>1.479848325507466</v>
       </c>
       <c r="U6" t="n">
-        <v>1.908528354104267</v>
+        <v>1.908547406669168</v>
       </c>
       <c r="V6" t="n">
-        <v>0.304557461770588</v>
+        <v>0.3045645988287349</v>
       </c>
       <c r="W6" t="n">
-        <v>-0.1977638642666655</v>
+        <v>-0.1977877785958579</v>
       </c>
       <c r="X6" t="n">
-        <v>0.2797509018709516</v>
+        <v>0.2797682235677406</v>
       </c>
       <c r="Y6" t="n">
-        <v>6.381102378142341</v>
+        <v>6.367708092874992</v>
       </c>
       <c r="Z6" t="n">
-        <v>6.583618469081034</v>
+        <v>6.555733993981558</v>
       </c>
       <c r="AA6" t="n">
-        <v>6.711995028099045</v>
+        <v>6.712311227725481</v>
       </c>
     </row>
     <row r="7">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E7" t="n">
         <v>14228</v>
@@ -1027,7 +1027,7 @@
         <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>14227</v>
+        <v>14228</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1044,13 +1044,13 @@
         <v>31048</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M7" t="n">
         <v>1.025</v>
       </c>
       <c r="N7" t="n">
-        <v>5.581147360652281</v>
+        <v>5.58107769890357</v>
       </c>
       <c r="O7" t="n">
         <v>10.01</v>
@@ -1059,37 +1059,37 @@
         <v>1.1435</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.567707221829661</v>
+        <v>5.567644159389283</v>
       </c>
       <c r="R7" t="n">
         <v>9.695129642606867</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.01344013882262098</v>
+        <v>-0.01343353951428771</v>
       </c>
       <c r="T7" t="n">
-        <v>1.167084647303406</v>
+        <v>1.167062970173387</v>
       </c>
       <c r="U7" t="n">
-        <v>1.510326062908891</v>
+        <v>1.51030237503732</v>
       </c>
       <c r="V7" t="n">
-        <v>0.5047558869009385</v>
+        <v>0.5047570197169796</v>
       </c>
       <c r="W7" t="n">
-        <v>0.05299615225730514</v>
+        <v>0.05298644135783115</v>
       </c>
       <c r="X7" t="n">
-        <v>0.5026066851421211</v>
+        <v>0.5026090514116928</v>
       </c>
       <c r="Y7" t="n">
-        <v>4.930685139429564</v>
+        <v>4.911901185076306</v>
       </c>
       <c r="Z7" t="n">
-        <v>5.00339928342277</v>
+        <v>4.992644984145779</v>
       </c>
       <c r="AA7" t="n">
-        <v>5.051737517240016</v>
+        <v>5.051723194369782</v>
       </c>
     </row>
     <row r="8">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E8" t="n">
         <v>9026</v>
@@ -1116,7 +1116,7 @@
         <v>10</v>
       </c>
       <c r="G8" t="n">
-        <v>9025</v>
+        <v>9026</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1133,13 +1133,13 @@
         <v>36161</v>
       </c>
       <c r="L8" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M8" t="n">
         <v>0.16</v>
       </c>
       <c r="N8" t="n">
-        <v>7.876887257617729</v>
+        <v>7.876636106802569</v>
       </c>
       <c r="O8" t="n">
         <v>15.14</v>
@@ -1148,37 +1148,37 @@
         <v>0.6453438395415473</v>
       </c>
       <c r="Q8" t="n">
-        <v>8.115837105028387</v>
+        <v>8.11542688243064</v>
       </c>
       <c r="R8" t="n">
         <v>14.26297827610371</v>
       </c>
       <c r="S8" t="n">
-        <v>0.2389498474106584</v>
+        <v>0.2387907756280712</v>
       </c>
       <c r="T8" t="n">
-        <v>1.446516052246957</v>
+        <v>1.446389343105706</v>
       </c>
       <c r="U8" t="n">
-        <v>1.826095366888119</v>
+        <v>1.825997102989003</v>
       </c>
       <c r="V8" t="n">
-        <v>0.807863206912252</v>
+        <v>0.8078809334385413</v>
       </c>
       <c r="W8" t="n">
-        <v>0.6274609164852973</v>
+        <v>0.6274834284506714</v>
       </c>
       <c r="X8" t="n">
-        <v>0.797853774270515</v>
+        <v>0.7978925286148745</v>
       </c>
       <c r="Y8" t="n">
-        <v>4.764292458331322</v>
+        <v>4.699703624013628</v>
       </c>
       <c r="Z8" t="n">
-        <v>4.994657804820511</v>
+        <v>4.952161304131803</v>
       </c>
       <c r="AA8" t="n">
-        <v>5.218376753554645</v>
+        <v>5.215031733135461</v>
       </c>
     </row>
     <row r="9">
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E9" t="n">
         <v>13891</v>
@@ -1205,7 +1205,7 @@
         <v>10</v>
       </c>
       <c r="G9" t="n">
-        <v>13890</v>
+        <v>13891</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1222,13 +1222,13 @@
         <v>31778</v>
       </c>
       <c r="L9" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M9" t="n">
         <v>0.06</v>
       </c>
       <c r="N9" t="n">
-        <v>7.611813354931606</v>
+        <v>7.611610215247283</v>
       </c>
       <c r="O9" t="n">
         <v>14.03</v>
@@ -1237,37 +1237,37 @@
         <v>0.409614576033637</v>
       </c>
       <c r="Q9" t="n">
-        <v>7.657392629727465</v>
+        <v>7.657158746563804</v>
       </c>
       <c r="R9" t="n">
         <v>13.66547972483708</v>
       </c>
       <c r="S9" t="n">
-        <v>0.04557927479586086</v>
+        <v>0.04554853131652175</v>
       </c>
       <c r="T9" t="n">
-        <v>1.494454068628206</v>
+        <v>1.494403474178203</v>
       </c>
       <c r="U9" t="n">
-        <v>1.942362115990856</v>
+        <v>1.942304635359889</v>
       </c>
       <c r="V9" t="n">
-        <v>0.7565871654135065</v>
+        <v>0.7566064381817833</v>
       </c>
       <c r="W9" t="n">
-        <v>0.5246896613534281</v>
+        <v>0.5247178987097768</v>
       </c>
       <c r="X9" t="n">
-        <v>0.7551787062391889</v>
+        <v>0.7552002780578599</v>
       </c>
       <c r="Y9" t="n">
-        <v>5.116181955096716</v>
+        <v>5.075627614234958</v>
       </c>
       <c r="Z9" t="n">
-        <v>5.263307288412771</v>
+        <v>5.237953993155882</v>
       </c>
       <c r="AA9" t="n">
-        <v>5.361600587371512</v>
+        <v>5.361939349474199</v>
       </c>
     </row>
     <row r="10">
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E10" t="n">
         <v>3737</v>
@@ -1326,37 +1326,37 @@
         <v>4.255</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.61705334931016</v>
+        <v>10.61693768093387</v>
       </c>
       <c r="R10" t="n">
         <v>14.31670311368574</v>
       </c>
       <c r="S10" t="n">
-        <v>0.3119916688177878</v>
+        <v>0.3118760004414978</v>
       </c>
       <c r="T10" t="n">
-        <v>2.052529428273189</v>
+        <v>2.052570776139774</v>
       </c>
       <c r="U10" t="n">
-        <v>2.698204420852664</v>
+        <v>2.698252311890559</v>
       </c>
       <c r="V10" t="n">
-        <v>0.356837871736162</v>
+        <v>0.3568505388140931</v>
       </c>
       <c r="W10" t="n">
-        <v>-0.1205267571512865</v>
+        <v>-0.1205665344677969</v>
       </c>
       <c r="X10" t="n">
-        <v>0.3364019047413548</v>
+        <v>0.3364327795021365</v>
       </c>
       <c r="Y10" t="n">
-        <v>9.490076015867068</v>
+        <v>9.489485571553459</v>
       </c>
       <c r="Z10" t="n">
-        <v>9.794306710035501</v>
+        <v>9.661028628929499</v>
       </c>
       <c r="AA10" t="n">
-        <v>10.92479894014703</v>
+        <v>9.983611807071936</v>
       </c>
     </row>
     <row r="11">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E11" t="n">
         <v>13832</v>
@@ -1383,7 +1383,7 @@
         <v>10</v>
       </c>
       <c r="G11" t="n">
-        <v>13831</v>
+        <v>13832</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1400,52 +1400,52 @@
         <v>31413</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M11" t="n">
         <v>0.438</v>
       </c>
       <c r="N11" t="n">
-        <v>5.243540561058492</v>
+        <v>5.24346873192597</v>
       </c>
       <c r="O11" t="n">
         <v>10.15</v>
       </c>
       <c r="P11" t="n">
-        <v>0.4579030837004405</v>
+        <v>0.4578686720469552</v>
       </c>
       <c r="Q11" t="n">
-        <v>5.2170371100722</v>
+        <v>5.216954819575744</v>
       </c>
       <c r="R11" t="n">
         <v>9.96782041998552</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.02650345098629179</v>
+        <v>-0.02651391235022364</v>
       </c>
       <c r="T11" t="n">
-        <v>1.161727306651721</v>
+        <v>1.161671624261001</v>
       </c>
       <c r="U11" t="n">
-        <v>1.483193481715616</v>
+        <v>1.483155592547925</v>
       </c>
       <c r="V11" t="n">
-        <v>0.4292594939922887</v>
+        <v>0.4292803833545303</v>
       </c>
       <c r="W11" t="n">
-        <v>-0.09227911487965712</v>
+        <v>-0.09226357518707506</v>
       </c>
       <c r="X11" t="n">
-        <v>0.4274502578848689</v>
+        <v>0.4274728698913296</v>
       </c>
       <c r="Y11" t="n">
-        <v>4.069848874204602</v>
+        <v>4.069658229395941</v>
       </c>
       <c r="Z11" t="n">
-        <v>4.607848468541699</v>
+        <v>4.420538537606477</v>
       </c>
       <c r="AA11" t="n">
-        <v>5.455567566903852</v>
+        <v>4.944805575935437</v>
       </c>
     </row>
     <row r="12">
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E12" t="n">
         <v>4150</v>
@@ -1472,7 +1472,7 @@
         <v>10</v>
       </c>
       <c r="G12" t="n">
-        <v>4149</v>
+        <v>4150</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1489,52 +1489,52 @@
         <v>41640</v>
       </c>
       <c r="L12" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M12" t="n">
         <v>2.195</v>
       </c>
       <c r="N12" t="n">
-        <v>7.472374909616775</v>
+        <v>7.471526144578314</v>
       </c>
       <c r="O12" t="n">
         <v>19.178</v>
       </c>
       <c r="P12" t="n">
-        <v>2.20511013215859</v>
+        <v>2.20509904622157</v>
       </c>
       <c r="Q12" t="n">
-        <v>7.645967740067685</v>
+        <v>7.645183705009093</v>
       </c>
       <c r="R12" t="n">
         <v>16.78633667621756</v>
       </c>
       <c r="S12" t="n">
-        <v>0.1735928304509096</v>
+        <v>0.1736575604307796</v>
       </c>
       <c r="T12" t="n">
-        <v>0.9135210157863671</v>
+        <v>0.9134262137001391</v>
       </c>
       <c r="U12" t="n">
-        <v>1.195486757749265</v>
+        <v>1.195377508698834</v>
       </c>
       <c r="V12" t="n">
-        <v>0.8314450999029892</v>
+        <v>0.8315527479393762</v>
       </c>
       <c r="W12" t="n">
-        <v>0.658256926424848</v>
+        <v>0.6584811761704317</v>
       </c>
       <c r="X12" t="n">
-        <v>0.8296724632923537</v>
+        <v>0.8297756434583377</v>
       </c>
       <c r="Y12" t="n">
-        <v>4.291847932012725</v>
+        <v>4.289780141476372</v>
       </c>
       <c r="Z12" t="n">
-        <v>4.447259244732281</v>
+        <v>4.382665142311696</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.261474665264195</v>
+        <v>5.194906292848363</v>
       </c>
     </row>
     <row r="13">
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E13" t="n">
         <v>6485</v>
@@ -1561,7 +1561,7 @@
         <v>10</v>
       </c>
       <c r="G13" t="n">
-        <v>6484</v>
+        <v>6485</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1578,13 +1578,13 @@
         <v>39083</v>
       </c>
       <c r="L13" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M13" t="n">
         <v>1.54</v>
       </c>
       <c r="N13" t="n">
-        <v>9.605567165330044</v>
+        <v>9.605054356206631</v>
       </c>
       <c r="O13" t="n">
         <v>16.215</v>
@@ -1593,37 +1593,37 @@
         <v>2.866674842326559</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.02653430527363</v>
+        <v>10.02611038346507</v>
       </c>
       <c r="R13" t="n">
         <v>16.20563653352021</v>
       </c>
       <c r="S13" t="n">
-        <v>0.4209671399435899</v>
+        <v>0.4210560272584442</v>
       </c>
       <c r="T13" t="n">
-        <v>1.691594796210649</v>
+        <v>1.691565516550389</v>
       </c>
       <c r="U13" t="n">
-        <v>2.150994788191994</v>
+        <v>2.150938320013887</v>
       </c>
       <c r="V13" t="n">
-        <v>0.8231844240901107</v>
+        <v>0.8231942593098103</v>
       </c>
       <c r="W13" t="n">
-        <v>0.648661523915858</v>
+        <v>0.6486712847590157</v>
       </c>
       <c r="X13" t="n">
-        <v>0.8104862542112194</v>
+        <v>0.8104959205077582</v>
       </c>
       <c r="Y13" t="n">
-        <v>8.095916956552648</v>
+        <v>7.734893971690662</v>
       </c>
       <c r="Z13" t="n">
-        <v>8.414631067479345</v>
+        <v>8.362380353842648</v>
       </c>
       <c r="AA13" t="n">
-        <v>8.504605235412651</v>
+        <v>8.524916901728622</v>
       </c>
     </row>
     <row r="14">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E14" t="n">
         <v>14072</v>
@@ -1650,7 +1650,7 @@
         <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>14071</v>
+        <v>14072</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1667,52 +1667,52 @@
         <v>30682</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M14" t="n">
         <v>0.26</v>
       </c>
       <c r="N14" t="n">
-        <v>8.129009132257835</v>
+        <v>8.12877043064241</v>
       </c>
       <c r="O14" t="n">
         <v>34.002</v>
       </c>
       <c r="P14" t="n">
-        <v>0.9075599608418992</v>
+        <v>0.9074492540963561</v>
       </c>
       <c r="Q14" t="n">
-        <v>8.199533929339131</v>
+        <v>8.199190564544491</v>
       </c>
       <c r="R14" t="n">
         <v>14.32</v>
       </c>
       <c r="S14" t="n">
-        <v>0.07052479708129507</v>
+        <v>0.07042013390208088</v>
       </c>
       <c r="T14" t="n">
-        <v>1.756791903163342</v>
+        <v>1.756619432989678</v>
       </c>
       <c r="U14" t="n">
-        <v>2.282800757222165</v>
+        <v>2.282651813681312</v>
       </c>
       <c r="V14" t="n">
-        <v>0.7808444975098474</v>
+        <v>0.7808808489690872</v>
       </c>
       <c r="W14" t="n">
-        <v>0.5653542535218699</v>
+        <v>0.5654091474027513</v>
       </c>
       <c r="X14" t="n">
-        <v>0.7804665355412211</v>
+        <v>0.7805052154884849</v>
       </c>
       <c r="Y14" t="n">
-        <v>5.182085354725964</v>
+        <v>5.170432952914561</v>
       </c>
       <c r="Z14" t="n">
-        <v>5.251798942180962</v>
+        <v>5.25723773084998</v>
       </c>
       <c r="AA14" t="n">
-        <v>5.333237217994927</v>
+        <v>5.541744903459582</v>
       </c>
     </row>
     <row r="15">
@@ -1730,7 +1730,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E15" t="n">
         <v>3099</v>
@@ -1768,40 +1768,40 @@
         <v>30.745</v>
       </c>
       <c r="P15" t="n">
-        <v>4.673348017621145</v>
+        <v>4.672531181217901</v>
       </c>
       <c r="Q15" t="n">
-        <v>11.82214649833608</v>
+        <v>11.82201569404232</v>
       </c>
       <c r="R15" t="n">
         <v>21.32952932657494</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.1417408846907007</v>
+        <v>-0.1418716889844631</v>
       </c>
       <c r="T15" t="n">
-        <v>2.052342338424996</v>
+        <v>2.052366965071088</v>
       </c>
       <c r="U15" t="n">
-        <v>2.697594903444394</v>
+        <v>2.6976156015866</v>
       </c>
       <c r="V15" t="n">
-        <v>0.7949867055369728</v>
+        <v>0.7949895836601116</v>
       </c>
       <c r="W15" t="n">
-        <v>0.6096092127111992</v>
+        <v>0.6096032218969221</v>
       </c>
       <c r="X15" t="n">
-        <v>0.7863342903167907</v>
+        <v>0.7863453492445148</v>
       </c>
       <c r="Y15" t="n">
-        <v>10.9146802566502</v>
+        <v>8.531783128446474</v>
       </c>
       <c r="Z15" t="n">
-        <v>11.47024104993337</v>
+        <v>11.22091764442863</v>
       </c>
       <c r="AA15" t="n">
-        <v>11.8986089989068</v>
+        <v>11.90285020159987</v>
       </c>
     </row>
     <row r="16">
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E16" t="n">
         <v>9835</v>
@@ -1828,7 +1828,7 @@
         <v>10</v>
       </c>
       <c r="G16" t="n">
-        <v>9834</v>
+        <v>9835</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1845,13 +1845,13 @@
         <v>35804</v>
       </c>
       <c r="L16" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M16" t="n">
         <v>0.26</v>
       </c>
       <c r="N16" t="n">
-        <v>8.363813199105145</v>
+        <v>8.363633858668022</v>
       </c>
       <c r="O16" t="n">
         <v>131.9</v>
@@ -1860,37 +1860,37 @@
         <v>0.5268935553946416</v>
       </c>
       <c r="Q16" t="n">
-        <v>8.624373071903522</v>
+        <v>8.624591243343799</v>
       </c>
       <c r="R16" t="n">
         <v>131.7868211440985</v>
       </c>
       <c r="S16" t="n">
-        <v>0.2605598727983763</v>
+        <v>0.2609573846757762</v>
       </c>
       <c r="T16" t="n">
-        <v>3.59225820027089</v>
+        <v>3.592455325325715</v>
       </c>
       <c r="U16" t="n">
-        <v>11.09231864172644</v>
+        <v>11.09189241294237</v>
       </c>
       <c r="V16" t="n">
-        <v>0.04171001288694214</v>
+        <v>0.04169598518806215</v>
       </c>
       <c r="W16" t="n">
-        <v>-0.6099354251380775</v>
+        <v>-0.6099687370268541</v>
       </c>
       <c r="X16" t="n">
-        <v>0.0250462350960402</v>
+        <v>0.02503176609892821</v>
       </c>
       <c r="Y16" t="n">
-        <v>11.67317419041749</v>
+        <v>11.6592702707897</v>
       </c>
       <c r="Z16" t="n">
-        <v>11.84462858314012</v>
+        <v>11.81562759604806</v>
       </c>
       <c r="AA16" t="n">
-        <v>12.29480447072659</v>
+        <v>12.28361682988293</v>
       </c>
     </row>
     <row r="17">
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E17" t="n">
         <v>2379</v>
@@ -1917,7 +1917,7 @@
         <v>10</v>
       </c>
       <c r="G17" t="n">
-        <v>2378</v>
+        <v>2379</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1934,52 +1934,52 @@
         <v>43252</v>
       </c>
       <c r="L17" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M17" t="n">
         <v>1</v>
       </c>
       <c r="N17" t="n">
-        <v>6.494915895710681</v>
+        <v>6.493152585119798</v>
       </c>
       <c r="O17" t="n">
         <v>12.23</v>
       </c>
       <c r="P17" t="n">
-        <v>1.416938325991189</v>
+        <v>1.416731474688188</v>
       </c>
       <c r="Q17" t="n">
-        <v>6.859011435850739</v>
+        <v>6.857310746336936</v>
       </c>
       <c r="R17" t="n">
         <v>12.15775235336712</v>
       </c>
       <c r="S17" t="n">
-        <v>0.3640955401400583</v>
+        <v>0.3641581612171373</v>
       </c>
       <c r="T17" t="n">
-        <v>2.019635178994044</v>
+        <v>2.019008986043468</v>
       </c>
       <c r="U17" t="n">
-        <v>2.555376646656593</v>
+        <v>2.554882684807781</v>
       </c>
       <c r="V17" t="n">
-        <v>0.5324572448836055</v>
+        <v>0.5329405079111519</v>
       </c>
       <c r="W17" t="n">
-        <v>0.04350561296634237</v>
+        <v>0.0445085575133638</v>
       </c>
       <c r="X17" t="n">
-        <v>0.5291037257120532</v>
+        <v>0.5295807142133513</v>
       </c>
       <c r="Y17" t="n">
-        <v>2.42901347388417</v>
+        <v>2.428812436852707</v>
       </c>
       <c r="Z17" t="n">
-        <v>3.109052148873424</v>
+        <v>3.187052261260365</v>
       </c>
       <c r="AA17" t="n">
-        <v>4.373651612063481</v>
+        <v>4.605098930410115</v>
       </c>
     </row>
     <row r="18">
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E18" t="n">
         <v>3238</v>
@@ -2006,7 +2006,7 @@
         <v>10</v>
       </c>
       <c r="G18" t="n">
-        <v>3237</v>
+        <v>3238</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -2023,13 +2023,13 @@
         <v>42370</v>
       </c>
       <c r="L18" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M18" t="n">
         <v>1.81</v>
       </c>
       <c r="N18" t="n">
-        <v>6.477426320667283</v>
+        <v>6.476630327362569</v>
       </c>
       <c r="O18" t="n">
         <v>18.492</v>
@@ -2038,37 +2038,37 @@
         <v>1.826106587712805</v>
       </c>
       <c r="Q18" t="n">
-        <v>6.671940610170693</v>
+        <v>6.671110435821966</v>
       </c>
       <c r="R18" t="n">
         <v>14.92762307692291</v>
       </c>
       <c r="S18" t="n">
-        <v>0.1945142895034078</v>
+        <v>0.1944801084593968</v>
       </c>
       <c r="T18" t="n">
-        <v>1.09866568198048</v>
+        <v>1.098342171488396</v>
       </c>
       <c r="U18" t="n">
-        <v>1.486918199494539</v>
+        <v>1.486701148993269</v>
       </c>
       <c r="V18" t="n">
-        <v>0.6058011176596961</v>
+        <v>0.6061048276803712</v>
       </c>
       <c r="W18" t="n">
-        <v>0.2263205890156228</v>
+        <v>0.2268625634243212</v>
       </c>
       <c r="X18" t="n">
-        <v>0.6029108188996035</v>
+        <v>0.6032193851918206</v>
       </c>
       <c r="Y18" t="n">
-        <v>3.065100466388778</v>
+        <v>3.064848621014697</v>
       </c>
       <c r="Z18" t="n">
-        <v>4.427640372361481</v>
+        <v>4.429689299343201</v>
       </c>
       <c r="AA18" t="n">
-        <v>5.851688262856731</v>
+        <v>5.678285833089822</v>
       </c>
     </row>
     <row r="19">
@@ -2086,7 +2086,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E19" t="n">
         <v>7192</v>
@@ -2095,7 +2095,7 @@
         <v>10</v>
       </c>
       <c r="G19" t="n">
-        <v>7191</v>
+        <v>7192</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2112,13 +2112,13 @@
         <v>37987</v>
       </c>
       <c r="L19" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M19" t="n">
         <v>0.04</v>
       </c>
       <c r="N19" t="n">
-        <v>10.33624794882492</v>
+        <v>10.33492477753059</v>
       </c>
       <c r="O19" t="n">
         <v>24.588</v>
@@ -2127,37 +2127,37 @@
         <v>3.790455501051156</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.12812323577417</v>
+        <v>11.12751651751246</v>
       </c>
       <c r="R19" t="n">
         <v>17.53862298528381</v>
       </c>
       <c r="S19" t="n">
-        <v>0.7918752869492509</v>
+        <v>0.792591739981868</v>
       </c>
       <c r="T19" t="n">
-        <v>2.0519559141632</v>
+        <v>2.052597835470644</v>
       </c>
       <c r="U19" t="n">
-        <v>2.775412154571399</v>
+        <v>2.776317554766227</v>
       </c>
       <c r="V19" t="n">
-        <v>0.7271211058638399</v>
+        <v>0.72713513573626</v>
       </c>
       <c r="W19" t="n">
-        <v>0.4709515563977114</v>
+        <v>0.4709902014429682</v>
       </c>
       <c r="X19" t="n">
-        <v>0.678529178107754</v>
+        <v>0.678402222556959</v>
       </c>
       <c r="Y19" t="n">
-        <v>7.373783103762445</v>
+        <v>7.328981900053581</v>
       </c>
       <c r="Z19" t="n">
-        <v>7.641359266893268</v>
+        <v>7.442825134818501</v>
       </c>
       <c r="AA19" t="n">
-        <v>9.483260125984224</v>
+        <v>7.596810587768807</v>
       </c>
     </row>
     <row r="20">
@@ -2175,7 +2175,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E20" t="n">
         <v>620</v>
@@ -2184,7 +2184,7 @@
         <v>10</v>
       </c>
       <c r="G20" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2201,52 +2201,52 @@
         <v>45658</v>
       </c>
       <c r="L20" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="M20" t="n">
-        <v>10.17</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="N20" t="n">
-        <v>15.53037964458805</v>
+        <v>15.52139516129032</v>
       </c>
       <c r="O20" t="n">
         <v>19.03</v>
       </c>
       <c r="P20" t="n">
-        <v>10.80578193832599</v>
+        <v>10.80560161408657</v>
       </c>
       <c r="Q20" t="n">
-        <v>16.36246131691289</v>
+        <v>16.35350743283659</v>
       </c>
       <c r="R20" t="n">
         <v>19.01911469282878</v>
       </c>
       <c r="S20" t="n">
-        <v>0.8320816723248445</v>
+        <v>0.8321122715462624</v>
       </c>
       <c r="T20" t="n">
-        <v>0.8853762187692525</v>
+        <v>0.8853214736124554</v>
       </c>
       <c r="U20" t="n">
-        <v>1.261488999175827</v>
+        <v>1.26093391953712</v>
       </c>
       <c r="V20" t="n">
-        <v>0.9375384673387651</v>
+        <v>0.9379701495268326</v>
       </c>
       <c r="W20" t="n">
-        <v>0.785665515605934</v>
+        <v>0.7869442802952729</v>
       </c>
       <c r="X20" t="n">
-        <v>0.9012171840144266</v>
+        <v>0.9016665886112374</v>
       </c>
       <c r="Y20" t="n">
-        <v>10.79127888241834</v>
+        <v>10.79176797337919</v>
       </c>
       <c r="Z20" t="n">
-        <v>10.80724653607479</v>
+        <v>10.82128739375457</v>
       </c>
       <c r="AA20" t="n">
-        <v>10.82395906754772</v>
+        <v>10.85966919563299</v>
       </c>
     </row>
     <row r="21">
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>16690</v>
+        <v>16691</v>
       </c>
       <c r="E21" t="n">
         <v>10237</v>
@@ -2305,37 +2305,37 @@
         <v>125.4</v>
       </c>
       <c r="Q21" t="n">
-        <v>130.9753584184409</v>
+        <v>130.9753771703504</v>
       </c>
       <c r="R21" t="n">
         <v>135.52</v>
       </c>
       <c r="S21" t="n">
-        <v>0.1045914945373727</v>
+        <v>0.1046102464468784</v>
       </c>
       <c r="T21" t="n">
-        <v>0.7976783616021335</v>
+        <v>0.7976929735280958</v>
       </c>
       <c r="U21" t="n">
-        <v>1.046341146593539</v>
+        <v>1.046356125737014</v>
       </c>
       <c r="V21" t="n">
-        <v>0.864915864325453</v>
+        <v>0.8649119350598818</v>
       </c>
       <c r="W21" t="n">
-        <v>0.7307660521977413</v>
+        <v>0.7307583435784013</v>
       </c>
       <c r="X21" t="n">
-        <v>0.8641736514562061</v>
+        <v>0.8641693103538335</v>
       </c>
       <c r="Y21" t="n">
-        <v>128.035504300431</v>
+        <v>128.0329518813868</v>
       </c>
       <c r="Z21" t="n">
-        <v>128.4669467051054</v>
+        <v>128.3418756637311</v>
       </c>
       <c r="AA21" t="n">
-        <v>129.6620647167807</v>
+        <v>129.5435815587171</v>
       </c>
     </row>
   </sheetData>
@@ -2404,22 +2404,22 @@
         <v>9043370</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E2" t="n">
         <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>7.373783103762445</v>
+        <v>7.328981900053581</v>
       </c>
       <c r="G2" t="n">
-        <v>7.641359266893268</v>
+        <v>7.442825134818503</v>
       </c>
       <c r="H2" t="n">
-        <v>9.483260125984224</v>
+        <v>7.596810587768807</v>
       </c>
     </row>
     <row r="3">
@@ -2432,22 +2432,22 @@
         <v>9036028</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>4.930685139429564</v>
+        <v>4.911901185076306</v>
       </c>
       <c r="G3" t="n">
-        <v>5.00339928342277</v>
+        <v>4.992644984145779</v>
       </c>
       <c r="H3" t="n">
-        <v>5.051737517240016</v>
+        <v>5.051723194369782</v>
       </c>
     </row>
     <row r="4">
@@ -2460,22 +2460,22 @@
         <v>9040208</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E4" t="n">
         <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>4.069848874204602</v>
+        <v>4.069658229395941</v>
       </c>
       <c r="G4" t="n">
-        <v>4.607848468541699</v>
+        <v>4.420538537606477</v>
       </c>
       <c r="H4" t="n">
-        <v>5.455567566903852</v>
+        <v>4.944805575935437</v>
       </c>
     </row>
     <row r="5">
@@ -2488,22 +2488,22 @@
         <v>9053555</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E5" t="n">
         <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>11.67317419041749</v>
+        <v>11.6592702707897</v>
       </c>
       <c r="G5" t="n">
-        <v>11.84462858314012</v>
+        <v>11.81562759604806</v>
       </c>
       <c r="H5" t="n">
-        <v>12.29480447072659</v>
+        <v>12.28361682988293</v>
       </c>
     </row>
     <row r="6">
@@ -2516,22 +2516,22 @@
         <v>9038134</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E6" t="n">
         <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>2.975828943454343</v>
+        <v>2.975681600135594</v>
       </c>
       <c r="G6" t="n">
-        <v>80.91433054852874</v>
+        <v>95.02088030319564</v>
       </c>
       <c r="H6" t="n">
-        <v>110.2664412526513</v>
+        <v>111.56</v>
       </c>
     </row>
     <row r="7">
@@ -2544,22 +2544,22 @@
         <v>9044756</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E7" t="n">
         <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>10.9146802566502</v>
+        <v>8.531783128446474</v>
       </c>
       <c r="G7" t="n">
-        <v>11.47024104993337</v>
+        <v>11.22091764442863</v>
       </c>
       <c r="H7" t="n">
-        <v>11.8986089989068</v>
+        <v>11.90285020159987</v>
       </c>
     </row>
     <row r="8">
@@ -2572,22 +2572,22 @@
         <v>9042214</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E8" t="n">
         <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>8.095916956552648</v>
+        <v>7.734893971690662</v>
       </c>
       <c r="G8" t="n">
-        <v>8.414631067479345</v>
+        <v>8.362380353842648</v>
       </c>
       <c r="H8" t="n">
-        <v>8.504605235412651</v>
+        <v>8.524916901728622</v>
       </c>
     </row>
     <row r="9">
@@ -2600,22 +2600,22 @@
         <v>9043597</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E9" t="n">
         <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>4.291847932012725</v>
+        <v>4.289780141476372</v>
       </c>
       <c r="G9" t="n">
-        <v>4.447259244732282</v>
+        <v>4.382665142311696</v>
       </c>
       <c r="H9" t="n">
-        <v>5.261474665264195</v>
+        <v>5.194906292848363</v>
       </c>
     </row>
     <row r="10">
@@ -2628,22 +2628,22 @@
         <v>9040454</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E10" t="n">
         <v>10</v>
       </c>
       <c r="F10" t="n">
-        <v>4.764292458331322</v>
+        <v>4.699703624013628</v>
       </c>
       <c r="G10" t="n">
-        <v>4.994657804820511</v>
+        <v>4.952161304131802</v>
       </c>
       <c r="H10" t="n">
-        <v>5.218376753554645</v>
+        <v>5.215031733135461</v>
       </c>
     </row>
     <row r="11">
@@ -2656,22 +2656,22 @@
         <v>9038835</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E11" t="n">
         <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>10.79127888241834</v>
+        <v>10.79176797337919</v>
       </c>
       <c r="G11" t="n">
-        <v>10.80724653607479</v>
+        <v>10.82128739375457</v>
       </c>
       <c r="H11" t="n">
-        <v>10.82395906754772</v>
+        <v>10.85966919563299</v>
       </c>
     </row>
     <row r="12">
@@ -2684,22 +2684,22 @@
         <v>9037610</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>2.42901347388417</v>
+        <v>2.428812436852707</v>
       </c>
       <c r="G12" t="n">
-        <v>3.109052148873424</v>
+        <v>3.187052261260365</v>
       </c>
       <c r="H12" t="n">
-        <v>4.373651612063481</v>
+        <v>4.605098930410115</v>
       </c>
     </row>
     <row r="13">
@@ -2712,22 +2712,22 @@
         <v>9043425</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E13" t="n">
         <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>5.182085354725964</v>
+        <v>5.170432952914561</v>
       </c>
       <c r="G13" t="n">
-        <v>5.251798942180962</v>
+        <v>5.25723773084998</v>
       </c>
       <c r="H13" t="n">
-        <v>5.333237217994927</v>
+        <v>5.541744903459582</v>
       </c>
     </row>
     <row r="14">
@@ -2740,22 +2740,22 @@
         <v>9042153</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E14" t="n">
         <v>10</v>
       </c>
       <c r="F14" t="n">
-        <v>9.490076015867068</v>
+        <v>9.489485571553459</v>
       </c>
       <c r="G14" t="n">
-        <v>9.794306710035503</v>
+        <v>9.6610286289295</v>
       </c>
       <c r="H14" t="n">
-        <v>10.92479894014703</v>
+        <v>9.983611807071936</v>
       </c>
     </row>
     <row r="15">
@@ -2768,22 +2768,22 @@
         <v>9040439</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
       </c>
       <c r="F15" t="n">
-        <v>5.116181955096716</v>
+        <v>5.075627614234958</v>
       </c>
       <c r="G15" t="n">
-        <v>5.263307288412771</v>
+        <v>5.237953993155882</v>
       </c>
       <c r="H15" t="n">
-        <v>5.361600587371512</v>
+        <v>5.361939349474199</v>
       </c>
     </row>
     <row r="16">
@@ -2796,22 +2796,22 @@
         <v>9032282</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E16" t="n">
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>6.381102378142341</v>
+        <v>6.367708092874992</v>
       </c>
       <c r="G16" t="n">
-        <v>6.583618469081034</v>
+        <v>6.555733993981558</v>
       </c>
       <c r="H16" t="n">
-        <v>6.711995028099045</v>
+        <v>6.712311227725481</v>
       </c>
     </row>
     <row r="17">
@@ -2824,22 +2824,22 @@
         <v>9037738</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E17" t="n">
         <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>3.065100466388778</v>
+        <v>3.064848621014697</v>
       </c>
       <c r="G17" t="n">
-        <v>4.427640372361481</v>
+        <v>4.429689299343201</v>
       </c>
       <c r="H17" t="n">
-        <v>5.851688262856731</v>
+        <v>5.678285833089822</v>
       </c>
     </row>
     <row r="18">
@@ -2852,22 +2852,22 @@
         <v>9039635</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E18" t="n">
         <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>3.181960352422907</v>
+        <v>3.180150403521643</v>
       </c>
       <c r="G18" t="n">
-        <v>3.304003187825538</v>
+        <v>3.456767148899859</v>
       </c>
       <c r="H18" t="n">
-        <v>3.496518272400334</v>
+        <v>3.968782098312546</v>
       </c>
     </row>
     <row r="19">
@@ -2880,22 +2880,22 @@
         <v>9038269</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E19" t="n">
         <v>10</v>
       </c>
       <c r="F19" t="n">
-        <v>2.150881791483113</v>
+        <v>2.089206338985151</v>
       </c>
       <c r="G19" t="n">
-        <v>2.225661007061721</v>
+        <v>2.207129567189043</v>
       </c>
       <c r="H19" t="n">
-        <v>2.331233021292217</v>
+        <v>2.330687820983126</v>
       </c>
     </row>
     <row r="20">
@@ -2908,22 +2908,22 @@
         <v>9036459</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E20" t="n">
         <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>4.871414572875782</v>
+        <v>4.776907411505261</v>
       </c>
       <c r="G20" t="n">
-        <v>5.19583926257148</v>
+        <v>5.194475984089943</v>
       </c>
       <c r="H20" t="n">
-        <v>5.726413692731685</v>
+        <v>5.807229304175822</v>
       </c>
     </row>
     <row r="21">
@@ -2936,22 +2936,22 @@
         <v>9046779</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E21" t="n">
         <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>128.035504300431</v>
+        <v>128.0329518813868</v>
       </c>
       <c r="G21" t="n">
-        <v>128.4669467051054</v>
+        <v>128.3418756637311</v>
       </c>
       <c r="H21" t="n">
-        <v>129.6620647167807</v>
+        <v>129.5435815587171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>